<commit_message>
docs(cambios): la planilla recoge los pendientes cerrados y la corrida de pruebas
Entran las seis cosas de esta tanda, salen los tres pendientes que se
decidieron, y la hoja de verificación cuenta el resultado real de la suite:
110 de 121, con las once que fallan comprobadas contra el código de ayer.
</commit_message>
<xml_diff>
--- a/docs/Control de cambios - Command Center.xlsx
+++ b/docs/Control de cambios - Command Center.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Verificación" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cambios'!$A$1:$H$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cambios'!$A$1:$H$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base de datos'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Productos creados'!$A$1:$E$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pendientes'!$A$1:$E$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Verificación'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pendientes'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Verificación'!$A$1:$C$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1364,37 +1364,289 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
+          <t>Borrar una venta también se cierra</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Solo el super admin puede borrar una venta registrada.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Con editar cerrado y borrar abierto, el bloqueo era un adorno: se borraba y se volvía a crear con otra cifra.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>2419a8f</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>La financiación mixta se declara en el catálogo</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>El catálogo de financiaciones dice cuáles son mixtas; el formulario ya no lo adivina por el nombre del código.</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Pedía el reparto si el código empezaba por «mixt»: se habría roto el día que alguien creara «Combinada».</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Nueva venta · catálogo</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>2419a8f</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Empresas</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Punto Tránsito estrena URL</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>De /e/tramites-buenaventura a /e/punto-transito.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>La URL decía otro nombre. Los enlaces viejos dejan de funcionar.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>URL de la empresa</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2419a8f</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>La suite aprende las reglas nuevas</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>La matriz de capacidades gana la marca «firmado» y las cuatro pruebas que afirmaban lo contrario comprueban lo que de verdad pasa.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Una prueba que afirma una regla derogada no avisa de nada: solo falla.</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>2419a8f</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Cinco pruebas que fallaban por cómo estaban escritas</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>El helper de guardar confundía los popover con el diálogo; tres buscaban un comercial que ya no se llama así; el alta de empresa escribía antes de que React hidratara; el borrado llegaba al menú por la forma del HTML.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Eran fallos de la prueba, no del software, y tapaban los de verdad.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2419a8f</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Cinco cuentas de prueba restauradas</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Los dos coordinadores y los tres asesores del plantel e2e, eliminados el 10/09, vuelven a entrar.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Sin ellas la suite no podía ni iniciar sesión: 13 pruebas morían antes de empezar.</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
           <t>La venta vieja conserva su precio</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Al abrir una venta ya registrada, el valor es el de esa venta y no el de la lista de hoy; si difieren, el formulario lo dice.</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Cambiar en silencio una cifra contra la que ya se liquidaron comisiones y se recibieron pagos.</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Editar venta</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Hecho</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>55778df</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H22"/>
+  <autoFilter ref="A1:H28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1923,7 +2175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1968,22 +2220,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Pruebas</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Borrar una venta sigue permitido al comercial</t>
+          <t>Siete pruebas de Usuarios fallan desde antes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>El bloqueo cierra editar, pero quien quiera cambiar una cifra puede borrar la venta y volverla a crear.</t>
+          <t>02-usuarios: el formulario de crear cuenta no encuentra «Crear e invitar» ni la opción «Editar y asignar empresas». Falla igual con el código de ayer, así que viene de antes.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Decidir si borrar también queda solo para el super admin.</t>
+          <t>Mirar si cambió el formulario de usuarios y las pruebas se quedaron atrás, o al revés.</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2247,22 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Productos</t>
+          <t>Pruebas</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Los precios generados hay que revisarlos</t>
+          <t>Tres pruebas de pantalla fallan desde antes</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Salieron del valor más repetido del último año de cada empresa; son un punto de partida, no la lista oficial.</t>
+          <t>Registrar un pago (la búsqueda de la venta no la encuentra), registrar una jornada y el importe de caja, que guarda −250.000 donde la prueba espera 250.000. Las tres fallan igual con el código de ayer.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Revisar empresa por empresa en la pantalla de Productos y corregir lo que esté mal.</t>
+          <t>Revisar una por una: la de caja huele a signo invertido de verdad.</t>
         </is>
       </c>
     </row>
@@ -2027,17 +2279,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Ningún producto tiene bonos todavía</t>
+          <t>Los precios generados hay que revisarlos</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Los bonos no se pueden deducir del histórico: el descuento venía en una columna suelta sin decir de qué bono era.</t>
+          <t>Salieron del valor más repetido del último año de cada empresa; son un punto de partida, no la lista oficial.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Cargarlos a mano por empresa.</t>
+          <t>Revisar empresa por empresa en la pantalla de Productos y corregir lo que esté mal.</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2301,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Productos</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>La financiación mixta se detecta por el nombre del código</t>
+          <t>Ningún producto tiene bonos todavía</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Las líneas aparecen cuando el tipo empieza por «mixt»; en el catálogo hay siete variantes.</t>
+          <t>Los bonos no se pueden deducir del histórico: el descuento venía en una columna suelta sin decir de qué bono era.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Marcar el catálogo de financiaciones en vez de adivinar por el nombre.</t>
+          <t>Cargarlos a mano por empresa.</t>
         </is>
       </c>
     </row>
@@ -2103,54 +2355,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Empresas</t>
+          <t>Ventas</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>El slug de Punto Tránsito sigue siendo tramites-buenaventura</t>
+          <t>10 ventas quedaron sin producto</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>La URL es /e/tramites-buenaventura. No se cambió para no romper enlaces guardados.</t>
+          <t>No traen código de producto o traen un número que se coló en la columna al importar.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Decidir si se cambia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Ventas</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>10 ventas quedaron sin producto</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>No traen código de producto o traen un número que se coló en la columna al importar.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
           <t>Asignarles producto a mano si importan.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:E7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2161,7 +2386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2296,17 +2521,34 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Se corrió contra el código nuevo. 13 pruebas fallan porque cinco cuentas de prueba (dos coordinadores y tres asesores) están eliminadas en Auth desde el 10/09 a las 15:07, un día antes de estos cambios: la prueba no llega ni a entrar. La única que corre con el super admin pasó.</t>
+          <t>121 pruebas contra el código nuevo: 110 pasan. Las 11 que fallan se comprobaron una por una contra el código de ayer en un árbol aparte: diez fallan igual sin ninguno de estos cambios y la otra solo falla cuando corre junto a las demás (ve las empresas de prueba que las otras están usando en ese momento).</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bloqueado por las cuentas, no por el código</t>
+          <t>OK · ningún fallo viene de estos cambios</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Nada de lo cambiado falla</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Ventas, productos, permisos en la base y aislamiento entre empresas: verde. Incluida la regla nueva —el coordinador no corrige ni borra una venta, el super admin sí— y que un asesor de pruebas no alcanza ni una venta del cliente.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C8"/>
+  <autoFilter ref="A1:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(cambios): la planilla recoge la jornada por bloques, la venta completa y los indicadores
Dieciséis cambios, la migración 044, seis verificaciones y las dudas que hay que confirmar con el cliente: venta externa, fórmula de facturación y metas mensuales. Y la nota de que la suite e2e no corrió porque falta .env.e2e en esta máquina.
</commit_message>
<xml_diff>
--- a/docs/Control de cambios - Command Center.xlsx
+++ b/docs/Control de cambios - Command Center.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cambios" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Base de datos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Productos creados" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Pendientes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Verificación" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cambios" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base de datos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos creados" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificación" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cambios'!$A$1:$H$28</definedName>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1645,6 +1645,678 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Gestión Diaria</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Registrar jornada por bloques, como el Excel</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Cinco bloques con título de color: Llamadas, Agendas, Atención venta presencial, Atención agenda, Atención administrativa, y la cola del CRM aparte. Cada bloque muestra su total al pie.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>El equipo llenaba el formulario mirando la hoja de Excel y las casillas planas no se correspondían con sus títulos.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Registrar jornada</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Gestión Diaria</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>«Contestadas» ya no se digita</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Es la suma de efectiva + seguimiento + agenda + no interesado + postventa. Aparecen «Total de llamadas» y «Total de agendas» calculados.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Cuando era una casilla, se llenaba a ojo y no cuadraba con el detalle; así se detectaron los errores.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Registrar jornada · Indicadores</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Gestión Diaria</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Las vistas contaban dos veces las contestadas</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Los totales de llamadas y contestadas de la 014 sumaban la columna «contestada» como una tipificación más. Se corrigió y se recalcularon 406 jornadas importadas que la traían mal.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>El ratio de contactabilidad salía inflado en todos los tableros.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard · Indicadores · base de datos</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Gestión Diaria</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Campo «Venta externa» en atención presencial</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo contador que suma al total de atención presencial y a las ventas presenciales de la gestión.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Lo pidió la gerencia el 11/09: no había dónde registrar la venta cerrada fuera del punto.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Registrar jornada</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Hecho · confirmar con el cliente si suma al total presencial</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Gestión Diaria</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Atención agenda no suma</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>«Agenda atendida» queda como dato suelto fuera de los totales.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>El mismo cliente que vino por agenda ya está contado como venta, seguimiento o declinado; sumarlo duplicaría personas.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Registrar jornada · Indicadores</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Tipo de venta presencial o digital</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Selector en el bloque «La venta». Es lo que se cruza contra la gestión diaria.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Sin él no se puede validar que el equipo tipifique igual en la base y en la gestión (KPI 1).</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Nueva venta</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Canal, categoría, tipo de documento, pagaré, voucher, contrato y examen médico</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Todos los campos de la hoja Base que faltaban en el formulario. El tipo de documento va tanto para el cliente como para el titular del crédito (arranca en CC).</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>La regla que dio el cliente: todo lo que está en la base tiene que poder llenarse en el Command Center.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Nueva venta</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Sin devolución, evento ni valor de lámina</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>No se agregaron esos campos.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Sales Trainer: siempre están en cero en el Excel, y la lámina va como adición.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Nueva venta</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Decidido</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Fotos del comprobante en la venta</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Una o varias fotos o PDF del pago, guardadas en el bucket privado de comprobantes bajo la carpeta de la empresa. Se ven al abrir la venta.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>El asesor tenía que ir al CRM a buscar el chat con el pago cada vez que había una duda.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Nueva venta</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Hecho · quitar una foto queda para el super admin</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Pantalla nueva de indicadores</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Los 14 KPI de la gerencia: cruce presencial/digital entre base y gestión, ratios con meta, logrado y efectividad, promedios, días laborados, tabla de totales por comercial y cantidad de ventas por tipo.</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Es el tablero que la gerencia arma hoy en Excel a mano.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>/e/{empresa}/indicadores</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Filtros de comerciales y de fecha</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Uno, varios o todos los comerciales; el período por mes, por día o por rango de fechas. Todo queda en la URL.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>«Poder hacer lo mismo que hago en Excel»: seleccionar a quién y cuándo, y que sume.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>/e/{empresa}/indicadores</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Días hábiles del mes configurables</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Campo junto a los filtros; lo fija quien administra. Contra ese número se mide el absentismo (meta 80 %).</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Julio tuvo 21 días hábiles; la cuenta fija de lunes a sábado no sirve.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>/e/{empresa}/indicadores</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Los totales los suma Postgres</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Función indicadores_por_comercial: una fila por comercial con gestión y ventas del rango. La pantalla solo rehace los ratios sobre lo filtrado.</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Las vistas mensuales no sirven para «del 3 al 17», y sumar en el navegador es la forma de que dos pantallas den cifras distintas.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Empresas</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Logo de Trámites Candelaria</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Cargado a Storage con el margen recortado.</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Lo mandó el cliente el 10/09.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Empresas · sidebar</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Logo de Genelypse Command Center en la entrada</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>La pantalla de inicio de sesión muestra el logo en vez del nombre en texto.</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Lo mandó el cliente el 10/09.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>/login</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Transcripción y requerimientos del feedback</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Los ocho videos transcritos y el documento de requerimientos con lo pedido, lo que había y las dudas por confirmar.</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Para no depender de volver a ver los videos.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>docs/feedback</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1657,7 +2329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1826,6 +2498,33 @@
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Precio = valor más repetido del último año. Se archiva lo que no se vende hace más de un año. El trigger de updated_at se apagó durante el enganche para no borrar el rastro de cuándo se tocó cada venta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>044</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>la_gestion_como_en_el_excel</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Contestadas derivada, venta externa, días hábiles por mes, fotos de la venta, vistas corregidas y la función del tablero de indicadores.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>daily_activity.atencion_venta_externa · company_business_days · sale_attachments · v_daily_activity · v_monthly_activity · v_branch_monthly · v_objective_progress · indicadores_por_comercial()</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Se recalcularon 406 jornadas cuya «contestada» no era la suma. El total de llamadas de la base pasó de 690.667 a 429.010 (ya no cuenta dos veces cada contestada). Sin avisos de seguridad nuevos.</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2333,12 +3032,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Cuatro empresas sin logo</t>
+          <t>Tres empresas sin logo</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>TTC, Trámites Candelaria, Trámites Florida y EMPRESA DE PRUEBA siguen con iniciales.</t>
+          <t>TTC, Trámites Florida y EMPRESA DE PRUEBA siguen con iniciales. Trámites Candelaria ya tiene el suyo.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2371,6 +3070,168 @@
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Asignarles producto a mano si importan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Gestión Diaria</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Confirmar con el cliente qué hace «venta externa»</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Se dejó sumando al total de atención presencial y a las ventas presenciales de la gestión.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Preguntar si va dentro del total presencial o aparte como «agenda atendida», y si en el KPI 1 cuenta como presencial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Fórmula de facturación total</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Se implementó como la dio la gerencia: valor final − (adición + descuento). Restar la adición deja la lámina fuera de la facturación.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Confirmar si es intencional o si la fórmula correcta es valor de lista − descuento + adición (que ya es el valor final).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Metas mensuales de 900 y 126</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>900 = 45 × 20 días y 126 = 6 × 21 días: se contradicen. El tablero mide la meta diaria (45 y 6) contra las jornadas registradas.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Confirmar que la lectura por jornada es la que quieren, o fijar un número de días para la mensual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>No se corrió la suite e2e</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Falta .env.e2e en esta máquina (las contraseñas del plantel). Se verificó a mano en local con capturas de pantalla.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Recuperar .env.e2e y correr `npx playwright test --grep "@gestion|@ventas"`. La prueba de jornada ya no rellena «ll-cont» porque ese campo no existe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Las ventas viejas no tienen tipo</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>16.539 ventas importadas traen sale_type_code; las que se registren sin elegir tipo salen como «sin tipo» en Indicadores.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Hacer obligatorio el tipo de venta si el cliente lo pide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Aviso de hidratación en /login</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Aparece de forma intermitente en la consola del navegador al abrir /login en desarrollo. No cambia nada visible.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Revisar SessionBounce o el indicador de desarrollo de Next.</t>
         </is>
       </c>
     </row>
@@ -2386,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2547,6 +3408,108 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Migración 044 aplicada</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Con el MCP de Supabase, en dos pasos (la función necesitó una condición de join por hash). Tipos de TypeScript regenerados.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>La contestada era la suma también en el Excel</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>9.549 de las 9.955 jornadas importadas traían «contestada» igual a la suma de las cinco tipificaciones; las otras 406 se recalcularon.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Compila y construye</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>TypeScript sin errores, ESLint sin errores nuevos (el único error es previo, en client-queries.ts) y build de producción completo con la ruta /indicadores.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Pantallas a mano en local</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Con la cuenta e2e «reserva» asignada temporalmente (y luego retirada): Registrar jornada con totales en vivo, Nueva venta con los campos nuevos, Indicadores de CEA la 28 en agosto de 2026 con datos reales, listado de Gestión Diaria y /login con el logo.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>OK · capturas revisadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>La función de indicadores cuadra</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CEA la 28, agosto 2026: 33 jornadas, 1.216 llamadas, 620 contestadas, 52 ventas (37 presenciales, 15 digitales); la gestión tipificó 28 presenciales y 18 efectivas.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>OK · la diferencia es justo lo que el KPI 1 quiere ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Avisos de seguridad de la base</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Las dos tablas nuevas tienen RLS y políticas; la función es security invoker y solo la llama authenticated. Sin hallazgos nuevos.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(cambios): la planilla recoge la venta a pantalla completa, las asesoras de Carss y la corrida e2e
</commit_message>
<xml_diff>
--- a/docs/Control de cambios - Command Center.xlsx
+++ b/docs/Control de cambios - Command Center.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2314,6 +2314,300 @@
       <c r="H44" s="2" t="inlineStr">
         <is>
           <t>ed64f3d</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>La venta a pantalla completa y en tres columnas</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Quién compra · qué compró · cómo la pagó. El diálogo ocupa toda la ventana.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Con doce bloques en 1.024 px había que bajar tres pantallas para llegar a la financiación.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Nueva venta · Editar venta</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>7ad219a</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Pagos</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Número de contrato</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Campo nuevo en el formulario de pago; la columna ya existía.</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Faltaba del Excel.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Registrar pago</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>7ad219a</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>El login ya no comprueba la sesión al cargar</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Se quitó el componente que hidrataba solo para redirigir si la sesión seguía viva.</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Daba avisos de hidratación y no aportaba: si la sesión venció, se vuelve a entrar y ya.</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>/login</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>7ad219a</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Ícono de la pestaña y de la tarjeta del sidebar</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>El símbolo de Genelypse reemplaza el triángulo de Next en la pestaña y las iniciales «CC» en la tarjeta sin empresa activa.</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Lo pidió el cliente con el logo.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Pestaña · sidebar</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>6797064</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Usuarios</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Asesoras de Carss (Cali)</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta nueva para Leidy Nataly Acevedo (nat.blue25@hotmail.com), asesora de Carss; a Ingrid Arias se le puso el celular. Acceso en ~/Downloads/accesos-carss.txt.</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Lo pidió el cliente en las notas de la reunión.</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Admin · Usuarios</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Hecho · la clave hay que dictársela</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Plantel e2e recuperado</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Se les puso contraseña nueva a las diez cuentas del plantel y se regeneró .env.e2e (no se versiona).</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Las cuentas se habían borrado y recreado sin contraseñas; la suite no podía ni entrar.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Cuatro pruebas corregidas</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>La fecha de hoy era la de Greenwich (fallaban desde las 7 pm); la jornada buscaba «responsable» en vez de «persona»; la búsqueda del pago no se enviaba; caja arrancaba en salida (negativo) y esperaba positivo.</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Eran fallos de la prueba, no del software.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>e2e</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>e8a62af</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3451,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -3167,17 +3461,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>No se corrió la suite e2e</t>
+          <t>La suite e2e corre, pero el Worker se queda sin CPU bajo carga</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Falta .env.e2e en esta máquina (las contraseñas del plantel). Se verificó a mano en local con capturas de pantalla.</t>
+          <t>Corrida completa: 102 de 121 pasan. Tras corregir cuatro pruebas, ventas y login pasan. Lo que sigue fallando: las 7 de Usuarios (de antes) y 03-empresas, 04-sedes, 09-pagos, 11-jornada y 12-caja, que mueren con «Worker exceeded resource limits» al entrar o al crear la empresa de prueba; el login a mano contra producción tarda 2,6 s y funciona.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Recuperar .env.e2e y correr `npx playwright test --grep "@gestion|@ventas"`. La prueba de jornada ya no rellena «ll-cont» porque ese campo no existe.</t>
+          <t>Revisar los límites de CPU del Worker (plan o tamaño del bundle) o correr la suite con --workers=1 fuera de horario. Y arreglar las 7 de Usuarios.</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3505,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -3226,12 +3520,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Aparece de forma intermitente en la consola del navegador al abrir /login en desarrollo. No cambia nada visible.</t>
+          <t>Resuelto: se quitó el componente que lo causaba (7ad219a).</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Revisar SessionBounce o el indicador de desarrollo de Next.</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3510,6 +3804,57 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Suite e2e contra producción</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>121 pruebas. Primera corrida 102 pasan; tras las cuatro correcciones, ventas (alta y edición) y login pasan. Las que quedan son las 7 de Usuarios (de antes) y las que el Worker rechaza por CPU.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Parcial · ver Pendientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Login en producción</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Entrar con la cuenta e2e super admin tarda 2,6 s y aterriza en /empresas.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Venta a pantalla completa</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Capturas a 1.440 y 1.920 px con una venta real de CEA la 28: tres columnas en pantallas anchas, dos en la mediana.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(cambios): la planilla recoge la versión móvil y su verificación
</commit_message>
<xml_diff>
--- a/docs/Control de cambios - Command Center.xlsx
+++ b/docs/Control de cambios - Command Center.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2608,6 +2608,48 @@
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>e8a62af</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>La app se abre en el celular</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Se quitó el aviso «Versión móvil no disponible»: el menú lateral se abre como panel desde el botón de la cabecera, los diálogos (venta, pago, jornada, agenda, caja, producto, sede, equipo) ocupan toda la pantalla, y la rejilla de Indicadores ya no se desborda por las tablas. Las tablas largas se desplazan de lado dentro de su tarjeta.</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Lo pidió el cliente: los comerciales registran desde el celular.</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Toda la app por debajo de 640 px</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>a506fe2</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3855,6 +3897,23 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Las 16 pantallas y 8 diálogos en celular</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Capturas con Playwright a 390 px (iPhone 14) entrando como super admin en Atenas: ninguna pantalla desborda el ancho; los diálogos muestran los botones sin scroll interno.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(indicadores): el tablero se lee como el Excel y cada empresa fija sus metas
De la revisión del 15 de septiembre (video y mensaje de la gerencia):

- Las tarjetas se tiñen enteras según el semáforo y llevan un chip que dice
  el estado en palabras: "Cumple", "Cerca de la meta", "Por debajo", "Sobre
  la meta", "Pasado del tope" o "Dato imposible". Dos rojos no significan lo
  mismo y el color solo no lo decía.
- Las metas dejan de estar clavadas en el código: quien administra la cambia
  en la propia tarjeta y queda en `company_kpi_targets` (migración 045).
  Sin fila rige la meta por defecto; vaciar el campo vuelve a ella.
- La tabla de totales usa los bloques y colores del formulario de la jornada.
  La cola del CRM lleva sus tres títulos (chats, tareas, caducadas) sobre
  "inicial · medio día · final": antes eran tres tríos iguales sin nombre.
- La distribución por canal (KPI 14) se ve: barra apilada y dos placas con
  la cifra grande.
</commit_message>
<xml_diff>
--- a/docs/Control de cambios - Command Center.xlsx
+++ b/docs/Control de cambios - Command Center.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2653,6 +2653,174 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Semáforo con más color y etiqueta</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Cada tarjeta se tiñe entera según su tono (verde cumple, ámbar cerca o sobre la meta, rojo lejos, pasado del tope o dato imposible), la efectividad va más grande y un chip dice el estado en palabras.</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Lo pidió la gerencia en el video del 15: con solo el número teñido, las diez tarjetas se veían iguales estuvieran bien o mal.</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores · Indicadores con meta</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Metas editables por empresa</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Quien administra cambia la meta de cada indicador en su tarjeta (70 → 50). Vacía vuelve a la meta por defecto. Se guarda en company_kpi_targets y queda en auditoría.</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>"Esas metas yo las puse porque son las actuales, pero pueden ser editables según la empresa."</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores · Indicadores con meta</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Totales por comercial como el Excel</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Bloques con el color del formulario de la jornada (llamadas azul, agendas verde, atención ámbar, cola del CRM violeta). La cola del CRM lleva ahora tres títulos (Chats, Tareas, Caducadas) sobre «Inicial · Medio día · Final», y atención presencial se divide en venta presencial, agenda y administrativa.</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>"Inicial, medio, final repetido tres veces… tendría que asumir que la primera es chats"; y que llamadas y agendas se distingan por color.</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores · Totales por comercial</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Distribución por canal más visual (KPI 14)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Barra apilada presencial/digital con el porcentaje encima y dos placas de color con la cifra grande.</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>"El KPI 14 no lo vi": estaba pero no se veía.</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores · Distribución de ventas por canal</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2665,7 +2833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2861,6 +3029,33 @@
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Se recalcularon 406 jornadas cuya «contestada» no era la suma. El total de llamadas de la base pasó de 690.667 a 429.010 (ya no cuenta dos veces cada contestada). Sin avisos de seguridad nuevos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>045</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>las_metas_son_de_cada_empresa</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>La meta de cada indicador del tablero, por empresa.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>company_kpi_targets (company_id, kpi_code, meta)</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Sin fila rige la meta por defecto del código. Ratios en fracción (0,7), cantidades tal cual (45). RLS igual que company_business_days. Sin avisos de seguridad nuevos.</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3914,6 +4109,57 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores con datos reales</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Carss, agosto 2026, entrando como super admin contra next dev: diez tarjetas coloreadas, tabla con bloques y tres niveles de encabezado, barra de reparto 56 % / 44 %. Sin errores de consola.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Meta editable de ida y vuelta</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Contactabilidad 70 → 50: al recargar sigue en 50 y la tarjeta pasa de «Por debajo» a «Cerca de la meta». Vaciar el campo la devuelve a 70 y borra la fila; la tabla quedó sin filas.</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Indicadores en celular</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>390 px: el documento mide 390 px de ancho, nada se desborda.</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>